<commit_message>
Several modifications on figures and scripts
</commit_message>
<xml_diff>
--- a/resultados/Relatorio_Comportamento_Por_Setor.xlsx
+++ b/resultados/Relatorio_Comportamento_Por_Setor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e124796\Gama_Workspace\ABMS-WP\resultados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{9B8A7B85-693C-4EAE-9B58-B8B2813DE28B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{A299C59C-51BD-48B8-93FB-265A187F4934}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{445F844C-0130-4D0C-B964-73D8B6288AE2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{445F844C-0130-4D0C-B964-73D8B6288AE2}"/>
   </bookViews>
   <sheets>
     <sheet name="Relatorio_Comportamento_Por_Set" sheetId="1" r:id="rId1"/>
@@ -1856,8 +1856,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39AB7FEC-3D38-437C-B2CD-4E81BFC0F26F}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:J68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
@@ -3789,8 +3803,8 @@
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
-  <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.78740157480314965" bottom="0.78740157480314965" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="88" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <headerFooter>
     <oddFooter>Página &amp;P de &amp;N</oddFooter>
   </headerFooter>

</xml_diff>